<commit_message>
#154 JLCPCB and Client BOM added.
</commit_message>
<xml_diff>
--- a/Design-Files/Electrode-Board-v4.0/EMG-Arm-ELEC-v1.0/Deliverables/BOM/Client-BOM-v1.0.xlsx
+++ b/Design-Files/Electrode-Board-v4.0/EMG-Arm-ELEC-v1.0/Deliverables/BOM/Client-BOM-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="119">
   <si>
     <t>#</t>
   </si>
@@ -90,21 +90,21 @@
     <t>J4</t>
   </si>
   <si>
-    <t>J16</t>
-  </si>
-  <si>
     <t>R1, R9, R24, R32, R37, R45, R50, R58, R63, R71, R76, R84, R89, R97, R102, R110</t>
   </si>
   <si>
     <t>R2, R7, R10, R12, R14, R15, R16, R18, R19, R20, R22, R23, R25, R30, R33, R35, R38, R43, R46, R48, R51, R56, R59, R61, R64, R69, R72, R74, R77, R82, R85, R87, R90, R95, R98, R100, R103, R108, R111, R113</t>
   </si>
   <si>
-    <t>R3, R4, R8, R26, R27, R31, R39, R40, R44, R52, R53, R57, R65, R66, R70, R78, R79, R83, R91, R92, R96, R104, R105, R109</t>
+    <t>R3, R4, R26, R27, R39, R40, R52, R53, R65, R66, R78, R79, R91, R92, R104, R105</t>
   </si>
   <si>
     <t>R5, R6, R11, R13, R17, R21, R28, R29, R34, R36, R41, R42, R47, R49, R54, R55, R60, R62, R67, R68, R73, R75, R80, R81, R86, R88, R93, R94, R99, R101, R106, R107, R112, R114</t>
   </si>
   <si>
+    <t>R8, R31, R44, R57, R70, R83, R96, R109</t>
+  </si>
+  <si>
     <t>R115, R116, R117, R118, R119, R120, R121</t>
   </si>
   <si>
@@ -162,12 +162,15 @@
     <t>RES 1K OHM 1% 1/16W 0402</t>
   </si>
   <si>
+    <t>RES 1M OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
+    <t>RES 10K OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
     <t>RES SMD 1M OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>RES 10K OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
     <t>RES 0 OHM JUMPER 1/10W 0603</t>
   </si>
   <si>
@@ -201,24 +204,18 @@
     <t>SOD323F</t>
   </si>
   <si>
-    <t>EMG 2 PAD</t>
+    <t>SEMG-PAD</t>
   </si>
   <si>
     <t>8.01A0.015200</t>
   </si>
   <si>
-    <t>EMG 3 Pad</t>
-  </si>
-  <si>
     <t>Res-0603</t>
   </si>
   <si>
     <t>Res-0402</t>
   </si>
   <si>
-    <t>TC-0522C-1.7-260G_</t>
-  </si>
-  <si>
     <t>SOT- 223</t>
   </si>
   <si>
@@ -264,12 +261,15 @@
     <t>RC0402FR-071KL</t>
   </si>
   <si>
+    <t>RC0402FR-071ML</t>
+  </si>
+  <si>
+    <t>RC0402FR-0710KL</t>
+  </si>
+  <si>
     <t>RC0603FR-071ML</t>
   </si>
   <si>
-    <t>RC0402FR-0710KL</t>
-  </si>
-  <si>
     <t>RC0603JR-070RL</t>
   </si>
   <si>
@@ -342,6 +342,9 @@
     <t>0.1uF</t>
   </si>
   <si>
+    <t>SEMG PAD</t>
+  </si>
+  <si>
     <t>1K</t>
   </si>
   <si>
@@ -357,19 +360,22 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
+    <t>DO NOT PLACE</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
     <t>Electrode Pad</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>DO NOT PLACE</t>
   </si>
 </sst>
 </file>
@@ -898,8 +904,7 @@
     <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -931,10 +936,10 @@
         <v>33</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H2" s="5" t="s">
         <v>88</v>
@@ -943,10 +948,10 @@
         <v>114</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -965,10 +970,10 @@
         <v>34</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>89</v>
@@ -997,10 +1002,10 @@
         <v>35</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>90</v>
@@ -1029,10 +1034,10 @@
         <v>36</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>90</v>
@@ -1061,10 +1066,10 @@
         <v>37</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>91</v>
@@ -1093,10 +1098,10 @@
         <v>38</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>90</v>
@@ -1125,13 +1130,13 @@
         <v>39</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H8" s="15" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="I8" s="16" t="s">
         <v>102</v>
@@ -1159,10 +1164,10 @@
         <v>40</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H9" s="7" t="s">
         <v>92</v>
@@ -1191,10 +1196,10 @@
         <v>41</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>91</v>
@@ -1223,10 +1228,10 @@
         <v>42</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>89</v>
@@ -1255,10 +1260,10 @@
         <v>35</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>92</v>
@@ -1287,16 +1292,16 @@
         <v>43</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>93</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="J13" s="7">
         <v>8</v>
@@ -1310,30 +1315,32 @@
         <v>12</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="D14" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="F14" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="H14" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="J14" s="9">
+      <c r="F14" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="I14" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="J14" s="15">
         <v>7</v>
       </c>
-      <c r="K14" s="9"/>
+      <c r="K14" s="17" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="15" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
@@ -1351,89 +1358,89 @@
         <v>45</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>94</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
       </c>
       <c r="K15" s="7"/>
     </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="11">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C16" s="13" t="s">
-        <v>113</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="C16" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="H16" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="I16" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="J16" s="9">
-        <v>1</v>
-      </c>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E16" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="I16" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="J16" s="15">
+        <v>16</v>
+      </c>
+      <c r="K16" s="17" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E17" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="F17" s="15" t="s">
-        <v>63</v>
-      </c>
-      <c r="G17" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="H17" s="15" t="s">
-        <v>112</v>
-      </c>
-      <c r="I17" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="J17" s="15">
-        <v>16</v>
-      </c>
-      <c r="K17" s="17" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E17" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="I17" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="J17" s="7">
+        <v>40</v>
+      </c>
+      <c r="K17" s="7"/>
+    </row>
+    <row r="18" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="11">
         <f t="shared" si="0"/>
@@ -1446,7 +1453,7 @@
         <v>25</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>64</v>
@@ -1458,30 +1465,30 @@
         <v>91</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="J18" s="9">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="K18" s="9"/>
     </row>
-    <row r="19" spans="1:11" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>26</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G19" s="8" t="s">
         <v>81</v>
@@ -1490,30 +1497,30 @@
         <v>91</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="J19" s="7">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="K19" s="7"/>
     </row>
-    <row r="20" spans="1:11" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="13" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>27</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G20" s="10" t="s">
         <v>82</v>
@@ -1525,7 +1532,7 @@
         <v>109</v>
       </c>
       <c r="J20" s="9">
-        <v>34</v>
+        <v>8</v>
       </c>
       <c r="K20" s="9"/>
     </row>
@@ -1542,7 +1549,7 @@
         <v>28</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>63</v>
@@ -1554,7 +1561,7 @@
         <v>91</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="J21" s="7">
         <v>7</v>
@@ -1574,10 +1581,10 @@
         <v>29</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>65</v>
+        <v>51</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>117</v>
       </c>
       <c r="G22" s="10" t="s">
         <v>84</v>
@@ -1586,7 +1593,7 @@
         <v>95</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="J22" s="9">
         <v>2</v>
@@ -1606,10 +1613,10 @@
         <v>30</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G23" s="8" t="s">
         <v>85</v>
@@ -1617,8 +1624,8 @@
       <c r="H23" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="I23" s="8" t="s">
-        <v>85</v>
+      <c r="I23" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="J23" s="7">
         <v>1</v>
@@ -1638,10 +1645,10 @@
         <v>31</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G24" s="10" t="s">
         <v>86</v>
@@ -1650,7 +1657,7 @@
         <v>96</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="J24" s="9">
         <v>8</v>
@@ -1670,10 +1677,10 @@
         <v>32</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>87</v>
@@ -1681,8 +1688,8 @@
       <c r="H25" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>87</v>
+      <c r="I25" s="10" t="s">
+        <v>115</v>
       </c>
       <c r="J25" s="7">
         <v>2</v>

</xml_diff>